<commit_message>
make final revisions to manuscript, format for gcb, and draft screening questions
</commit_message>
<xml_diff>
--- a/data/CNP_data_compiled_metadata.xlsx
+++ b/data/CNP_data_compiled_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eaperkowski/git/p_meta/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C155982E-514D-AC4A-9C2E-DA17E022F738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96CEE43E-A94F-CC44-8866-FB80F5DCFA08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="53100" yWindow="960" windowWidth="27640" windowHeight="16940" xr2:uid="{80CE26D0-6780-1444-B03C-08089C6B888D}"/>
+    <workbookView xWindow="1620" yWindow="5840" windowWidth="29000" windowHeight="18980" xr2:uid="{80CE26D0-6780-1444-B03C-08089C6B888D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="84">
   <si>
     <t>description</t>
   </si>
   <si>
-    <t>paper citation</t>
-  </si>
-  <si>
     <t>response variable</t>
   </si>
   <si>
@@ -59,27 +56,6 @@
     <t>latitude (in decimal degrees)</t>
   </si>
   <si>
-    <t>longitude (in decim</t>
-  </si>
-  <si>
-    <t>elevation</t>
-  </si>
-  <si>
-    <t>mean annual growing season precipitation</t>
-  </si>
-  <si>
-    <t>mean annual growing season potential evapotranspiration</t>
-  </si>
-  <si>
-    <t>mean annual growing season temperature</t>
-  </si>
-  <si>
-    <t>mean annual growing season aridity index</t>
-  </si>
-  <si>
-    <t>mean annual growing season PAR</t>
-  </si>
-  <si>
     <t>ecosystem type</t>
   </si>
   <si>
@@ -107,12 +83,6 @@
     <t>mycorrhizal association (from Soudzilovskaia 2019)</t>
   </si>
   <si>
-    <t>treatment (fnp = fertilization exp with n and p addition)</t>
-  </si>
-  <si>
-    <t>nutrient treatment (_100 = N, _010 = P, _110 = NP</t>
-  </si>
-  <si>
     <t>categorical fertilization description</t>
   </si>
   <si>
@@ -179,9 +149,6 @@
     <t>gs_map</t>
   </si>
   <si>
-    <t>gs_mapet</t>
-  </si>
-  <si>
     <t>gs_mat</t>
   </si>
   <si>
@@ -263,16 +230,64 @@
     <t>rep_t</t>
   </si>
   <si>
-    <t>x_units</t>
-  </si>
-  <si>
-    <t>units of trait</t>
-  </si>
-  <si>
     <t>doi</t>
   </si>
   <si>
     <t>url to paper</t>
+  </si>
+  <si>
+    <t>nutrient treatment (_100 = N, _010 = P, _110 = NP)</t>
+  </si>
+  <si>
+    <t>background_n_mgkg</t>
+  </si>
+  <si>
+    <t>bulk soil N content (mg/kg). 0-15cm depth from soilGrids</t>
+  </si>
+  <si>
+    <t>olsenP_mgkg</t>
+  </si>
+  <si>
+    <t>soil P availability (Olsen-P) from McDowell et al. (2023)</t>
+  </si>
+  <si>
+    <t>dataset_column</t>
+  </si>
+  <si>
+    <t>original source (mesi, nutnet, eap)</t>
+  </si>
+  <si>
+    <t>paper citation ([firstauthor][year])</t>
+  </si>
+  <si>
+    <t>longitude (in decimal degrees)</t>
+  </si>
+  <si>
+    <t>z</t>
+  </si>
+  <si>
+    <t>elevation (m)</t>
+  </si>
+  <si>
+    <t>growing season mean annual temperature (degC)</t>
+  </si>
+  <si>
+    <t>growing season mean annual preciptiation (mm)</t>
+  </si>
+  <si>
+    <t>growing season mean annual light availability (umol/m2/s)</t>
+  </si>
+  <si>
+    <t>growing season aridity index (unitless)</t>
+  </si>
+  <si>
+    <t>myc_nas</t>
+  </si>
+  <si>
+    <t>mycorrhizal nutrient acquisition strategy (from Cheaib et al. 2025)</t>
+  </si>
+  <si>
+    <t>treatment (fnp = fertilization exp with n and p addition, fp = p addition only)</t>
   </si>
 </sst>
 </file>
@@ -644,7 +659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90504DC5-F499-BB4C-B0A4-046292964F86}">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -654,7 +669,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -662,31 +677,31 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -694,290 +709,306 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="B33" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="B35" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B38" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B40" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B41" t="s">
-        <v>78</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>